<commit_message>
Add dev-filings-only corpus runs to Excel log and Task #5 doc
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Task #7_ Logging Runs.xlsx
+++ b/Task #7_ Logging Runs.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -332,7 +332,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Z13"/>
+  <dimension ref="A1:Z25"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <sheetData>
     <row r="1">
@@ -1328,6 +1328,898 @@
       <c r="S13" s="3" t="inlineStr">
         <is>
           <t>Development questions only; frozen test IDs excluded. Context header removed from chunker (no measurable benefit).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="4" t="n">
+        <v>46326</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Maanveer</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>85ef7ff</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Dev</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>48</v>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>Page</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>1 page</t>
+        </is>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="L14" s="3" t="inlineStr">
+        <is>
+          <t>TF-IDF</t>
+        </is>
+      </c>
+      <c r="M14" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="N14" s="3" t="n">
+        <v>0.021</v>
+      </c>
+      <c r="O14" s="3" t="n">
+        <v>0.167</v>
+      </c>
+      <c r="P14" s="3" t="n">
+        <v>0.188</v>
+      </c>
+      <c r="Q14" s="3" t="n">
+        <v>0.094</v>
+      </c>
+      <c r="R14" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="S14" s="3" t="inlineStr">
+        <is>
+          <t>Corpus changed: test filings removed, dev filings only (12 filings), so all runs re-evaluated. Matches CSV run 31.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="4" t="n">
+        <v>46326</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Maanveer</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>85ef7ff</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Dev</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="n">
+        <v>48</v>
+      </c>
+      <c r="G15" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>Page</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>1 page</t>
+        </is>
+      </c>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="K15" s="3" t="inlineStr">
+        <is>
+          <t>On</t>
+        </is>
+      </c>
+      <c r="L15" s="3" t="inlineStr">
+        <is>
+          <t>TF-IDF</t>
+        </is>
+      </c>
+      <c r="M15" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="N15" s="3" t="n">
+        <v>0.021</v>
+      </c>
+      <c r="O15" s="3" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="P15" s="3" t="n">
+        <v>0.271</v>
+      </c>
+      <c r="Q15" s="3" t="n">
+        <v>0.128</v>
+      </c>
+      <c r="R15" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="S15" s="3" t="inlineStr">
+        <is>
+          <t>Corpus changed: test filings removed, dev filings only (12 filings), so all runs re-evaluated. Matches CSV run 32.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="4" t="n">
+        <v>46326</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Maanveer</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>85ef7ff</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Dev</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="n">
+        <v>48</v>
+      </c>
+      <c r="G16" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>Words</t>
+        </is>
+      </c>
+      <c r="I16" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="J16" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="K16" s="3" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="L16" s="3" t="inlineStr">
+        <is>
+          <t>TF-IDF</t>
+        </is>
+      </c>
+      <c r="M16" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="N16" s="3" t="n">
+        <v>0.062</v>
+      </c>
+      <c r="O16" s="3" t="n">
+        <v>0.188</v>
+      </c>
+      <c r="P16" s="3" t="n">
+        <v>0.146</v>
+      </c>
+      <c r="Q16" s="3" t="n">
+        <v>0.112</v>
+      </c>
+      <c r="R16" s="3" t="n">
+        <v>0.958</v>
+      </c>
+      <c r="S16" s="3" t="inlineStr">
+        <is>
+          <t>Corpus changed: test filings removed, dev filings only (12 filings), so all runs re-evaluated. Matches CSV run 33.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="4" t="n">
+        <v>46326</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Maanveer</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>85ef7ff</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Dev</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="n">
+        <v>48</v>
+      </c>
+      <c r="G17" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>Words</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="J17" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="K17" s="3" t="inlineStr">
+        <is>
+          <t>On</t>
+        </is>
+      </c>
+      <c r="L17" s="3" t="inlineStr">
+        <is>
+          <t>TF-IDF</t>
+        </is>
+      </c>
+      <c r="M17" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="N17" s="3" t="n">
+        <v>0.083</v>
+      </c>
+      <c r="O17" s="3" t="n">
+        <v>0.229</v>
+      </c>
+      <c r="P17" s="3" t="n">
+        <v>0.208</v>
+      </c>
+      <c r="Q17" s="3" t="n">
+        <v>0.162</v>
+      </c>
+      <c r="R17" s="3" t="n">
+        <v>0.958</v>
+      </c>
+      <c r="S17" s="3" t="inlineStr">
+        <is>
+          <t>Corpus changed: test filings removed, dev filings only (12 filings), so all runs re-evaluated. Matches CSV run 34.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="4" t="n">
+        <v>46326</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Maanveer</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>85ef7ff</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>Dev</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="n">
+        <v>48</v>
+      </c>
+      <c r="G18" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>Words</t>
+        </is>
+      </c>
+      <c r="I18" s="3" t="n">
+        <v>600</v>
+      </c>
+      <c r="J18" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="K18" s="3" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="L18" s="3" t="inlineStr">
+        <is>
+          <t>TF-IDF</t>
+        </is>
+      </c>
+      <c r="M18" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="N18" s="3" t="n">
+        <v>0.042</v>
+      </c>
+      <c r="O18" s="3" t="n">
+        <v>0.167</v>
+      </c>
+      <c r="P18" s="3" t="n">
+        <v>0.208</v>
+      </c>
+      <c r="Q18" s="3" t="n">
+        <v>0.107</v>
+      </c>
+      <c r="R18" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="S18" s="3" t="inlineStr">
+        <is>
+          <t>Corpus changed: test filings removed, dev filings only (12 filings), so all runs re-evaluated. Matches CSV run 35.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="4" t="n">
+        <v>46326</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Maanveer</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>85ef7ff</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Dev</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="n">
+        <v>48</v>
+      </c>
+      <c r="G19" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>Words</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="n">
+        <v>600</v>
+      </c>
+      <c r="J19" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="K19" s="3" t="inlineStr">
+        <is>
+          <t>On</t>
+        </is>
+      </c>
+      <c r="L19" s="3" t="inlineStr">
+        <is>
+          <t>TF-IDF</t>
+        </is>
+      </c>
+      <c r="M19" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="N19" s="3" t="n">
+        <v>0.042</v>
+      </c>
+      <c r="O19" s="3" t="n">
+        <v>0.229</v>
+      </c>
+      <c r="P19" s="3" t="n">
+        <v>0.271</v>
+      </c>
+      <c r="Q19" s="3" t="n">
+        <v>0.149</v>
+      </c>
+      <c r="R19" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="S19" s="3" t="inlineStr">
+        <is>
+          <t>Corpus changed: test filings removed, dev filings only (12 filings), so all runs re-evaluated. Matches CSV run 36.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="4" t="n">
+        <v>46326</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Maanveer</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>85ef7ff</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Dev</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="n">
+        <v>48</v>
+      </c>
+      <c r="G20" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>Page</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>1 page</t>
+        </is>
+      </c>
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="K20" s="3" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="L20" s="3" t="inlineStr">
+        <is>
+          <t>BM25</t>
+        </is>
+      </c>
+      <c r="M20" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="N20" s="3" t="n">
+        <v>0.188</v>
+      </c>
+      <c r="O20" s="3" t="n">
+        <v>0.354</v>
+      </c>
+      <c r="P20" s="3" t="n">
+        <v>0.396</v>
+      </c>
+      <c r="Q20" s="3" t="n">
+        <v>0.251</v>
+      </c>
+      <c r="R20" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="S20" s="3" t="inlineStr">
+        <is>
+          <t>Corpus changed: test filings removed, dev filings only (12 filings), so all runs re-evaluated. Matches CSV run 37.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="4" t="n">
+        <v>46326</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Maanveer</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>85ef7ff</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>Dev</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="n">
+        <v>48</v>
+      </c>
+      <c r="G21" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>Page</t>
+        </is>
+      </c>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>1 page</t>
+        </is>
+      </c>
+      <c r="J21" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="K21" s="3" t="inlineStr">
+        <is>
+          <t>On</t>
+        </is>
+      </c>
+      <c r="L21" s="3" t="inlineStr">
+        <is>
+          <t>BM25</t>
+        </is>
+      </c>
+      <c r="M21" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="N21" s="3" t="n">
+        <v>0.229</v>
+      </c>
+      <c r="O21" s="3" t="n">
+        <v>0.479</v>
+      </c>
+      <c r="P21" s="3" t="n">
+        <v>0.542</v>
+      </c>
+      <c r="Q21" s="3" t="n">
+        <v>0.322</v>
+      </c>
+      <c r="R21" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="S21" s="3" t="inlineStr">
+        <is>
+          <t>Corpus changed: test filings removed, dev filings only (12 filings), so all runs re-evaluated. Matches CSV run 38.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="4" t="n">
+        <v>46326</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Maanveer</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>85ef7ff</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>Dev</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="n">
+        <v>48</v>
+      </c>
+      <c r="G22" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>Words</t>
+        </is>
+      </c>
+      <c r="I22" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="J22" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="K22" s="3" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="L22" s="3" t="inlineStr">
+        <is>
+          <t>BM25</t>
+        </is>
+      </c>
+      <c r="M22" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="N22" s="3" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="O22" s="3" t="n">
+        <v>0.354</v>
+      </c>
+      <c r="P22" s="3" t="n">
+        <v>0.292</v>
+      </c>
+      <c r="Q22" s="3" t="n">
+        <v>0.218</v>
+      </c>
+      <c r="R22" s="3" t="n">
+        <v>0.958</v>
+      </c>
+      <c r="S22" s="3" t="inlineStr">
+        <is>
+          <t>Corpus changed: test filings removed, dev filings only (12 filings), so all runs re-evaluated. Matches CSV run 39.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="4" t="n">
+        <v>46326</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Maanveer</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>85ef7ff</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>Dev</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="n">
+        <v>48</v>
+      </c>
+      <c r="G23" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>Words</t>
+        </is>
+      </c>
+      <c r="I23" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="J23" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="K23" s="3" t="inlineStr">
+        <is>
+          <t>On</t>
+        </is>
+      </c>
+      <c r="L23" s="3" t="inlineStr">
+        <is>
+          <t>BM25</t>
+        </is>
+      </c>
+      <c r="M23" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="N23" s="3" t="n">
+        <v>0.167</v>
+      </c>
+      <c r="O23" s="3" t="n">
+        <v>0.438</v>
+      </c>
+      <c r="P23" s="3" t="n">
+        <v>0.354</v>
+      </c>
+      <c r="Q23" s="3" t="n">
+        <v>0.286</v>
+      </c>
+      <c r="R23" s="3" t="n">
+        <v>0.958</v>
+      </c>
+      <c r="S23" s="3" t="inlineStr">
+        <is>
+          <t>Corpus changed: test filings removed, dev filings only (12 filings), so all runs re-evaluated. Matches CSV run 40.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="4" t="n">
+        <v>46326</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>Maanveer</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>85ef7ff</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>Dev</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="n">
+        <v>48</v>
+      </c>
+      <c r="G24" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>Words</t>
+        </is>
+      </c>
+      <c r="I24" s="3" t="n">
+        <v>600</v>
+      </c>
+      <c r="J24" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="K24" s="3" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="L24" s="3" t="inlineStr">
+        <is>
+          <t>BM25</t>
+        </is>
+      </c>
+      <c r="M24" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="N24" s="3" t="n">
+        <v>0.188</v>
+      </c>
+      <c r="O24" s="3" t="n">
+        <v>0.354</v>
+      </c>
+      <c r="P24" s="3" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="Q24" s="3" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="R24" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="S24" s="3" t="inlineStr">
+        <is>
+          <t>Corpus changed: test filings removed, dev filings only (12 filings), so all runs re-evaluated. Matches CSV run 41.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="4" t="n">
+        <v>46326</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Maanveer</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>85ef7ff</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>Dev</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="n">
+        <v>48</v>
+      </c>
+      <c r="G25" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>Words</t>
+        </is>
+      </c>
+      <c r="I25" s="3" t="n">
+        <v>600</v>
+      </c>
+      <c r="J25" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="K25" s="3" t="inlineStr">
+        <is>
+          <t>On</t>
+        </is>
+      </c>
+      <c r="L25" s="3" t="inlineStr">
+        <is>
+          <t>BM25</t>
+        </is>
+      </c>
+      <c r="M25" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="N25" s="3" t="n">
+        <v>0.229</v>
+      </c>
+      <c r="O25" s="3" t="n">
+        <v>0.479</v>
+      </c>
+      <c r="P25" s="3" t="n">
+        <v>0.521</v>
+      </c>
+      <c r="Q25" s="3" t="n">
+        <v>0.316</v>
+      </c>
+      <c r="R25" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="S25" s="3" t="inlineStr">
+        <is>
+          <t>Corpus changed: test filings removed, dev filings only (12 filings), so all runs re-evaluated. Matches CSV run 42.</t>
         </is>
       </c>
     </row>

</xml_diff>